<commit_message>
use summit_date month, not departure date month
</commit_message>
<xml_diff>
--- a/web/flask/static/annual_report_template.xlsx
+++ b/web/flask/static/annual_report_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\apps\climberdb\git\web\flask\static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ABE8CC8-E191-4D3A-8C80-1749A39B9F80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D332130-0012-4C53-82F4-290A1EC0F289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2342,6 +2342,63 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="9" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -2354,12 +2411,6 @@
     <xf numFmtId="0" fontId="21" fillId="9" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="21" fillId="9" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -2372,27 +2423,6 @@
     <xf numFmtId="0" fontId="19" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="10" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2411,36 +2441,6 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2459,6 +2459,24 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2492,24 +2510,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2522,9 +2522,6 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2538,6 +2535,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -2843,24 +2843,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="61.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="296" t="s">
+      <c r="A1" s="273" t="s">
         <v>325</v>
       </c>
-      <c r="B1" s="297"/>
-      <c r="C1" s="297"/>
-      <c r="D1" s="297"/>
-      <c r="E1" s="297"/>
-      <c r="F1" s="298"/>
+      <c r="B1" s="274"/>
+      <c r="C1" s="274"/>
+      <c r="D1" s="274"/>
+      <c r="E1" s="274"/>
+      <c r="F1" s="275"/>
     </row>
     <row r="2" spans="1:6" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="299" t="s">
+      <c r="A2" s="276" t="s">
         <v>290</v>
       </c>
-      <c r="B2" s="300"/>
-      <c r="C2" s="300"/>
-      <c r="D2" s="300"/>
-      <c r="E2" s="300"/>
-      <c r="F2" s="301"/>
+      <c r="B2" s="277"/>
+      <c r="C2" s="277"/>
+      <c r="D2" s="277"/>
+      <c r="E2" s="277"/>
+      <c r="F2" s="278"/>
     </row>
     <row r="3" spans="1:6" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="229" t="s">
@@ -2881,32 +2881,32 @@
       <c r="F4" s="261"/>
     </row>
     <row r="5" spans="1:6" ht="24.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="287"/>
-      <c r="B5" s="288"/>
-      <c r="C5" s="288"/>
+      <c r="A5" s="283"/>
+      <c r="B5" s="284"/>
+      <c r="C5" s="284"/>
       <c r="D5" s="217"/>
       <c r="E5" s="218"/>
       <c r="F5" s="219"/>
     </row>
     <row r="6" spans="1:6" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="285" t="s">
+      <c r="A6" s="289" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="286"/>
-      <c r="C6" s="286"/>
+      <c r="B6" s="290"/>
+      <c r="C6" s="290"/>
       <c r="D6" s="220"/>
       <c r="E6" s="221"/>
       <c r="F6" s="221"/>
     </row>
     <row r="7" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="283" t="s">
+      <c r="A7" s="287" t="s">
         <v>291</v>
       </c>
-      <c r="B7" s="284"/>
-      <c r="C7" s="284"/>
-      <c r="D7" s="277"/>
-      <c r="E7" s="278"/>
-      <c r="F7" s="278"/>
+      <c r="B7" s="288"/>
+      <c r="C7" s="288"/>
+      <c r="D7" s="279"/>
+      <c r="E7" s="280"/>
+      <c r="F7" s="280"/>
     </row>
     <row r="8" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="241" t="s">
@@ -2945,19 +2945,19 @@
       <c r="F10" s="18"/>
     </row>
     <row r="11" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="287"/>
-      <c r="B11" s="288"/>
-      <c r="C11" s="288"/>
+      <c r="A11" s="283"/>
+      <c r="B11" s="284"/>
+      <c r="C11" s="284"/>
       <c r="D11" s="210"/>
       <c r="E11" s="18"/>
       <c r="F11" s="18"/>
     </row>
     <row r="12" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="304" t="s">
+      <c r="A12" s="286" t="s">
         <v>231</v>
       </c>
-      <c r="B12" s="304"/>
-      <c r="C12" s="304"/>
+      <c r="B12" s="286"/>
+      <c r="C12" s="286"/>
       <c r="D12" s="210"/>
       <c r="E12" s="18"/>
       <c r="F12" s="18"/>
@@ -2981,22 +2981,22 @@
       <c r="F14" s="51"/>
     </row>
     <row r="15" spans="1:6" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="287"/>
-      <c r="B15" s="288"/>
-      <c r="C15" s="288"/>
+      <c r="A15" s="283"/>
+      <c r="B15" s="284"/>
+      <c r="C15" s="284"/>
       <c r="D15" s="223"/>
       <c r="E15" s="224"/>
       <c r="F15" s="224"/>
     </row>
     <row r="16" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="283" t="s">
+      <c r="A16" s="287" t="s">
         <v>296</v>
       </c>
-      <c r="B16" s="305"/>
-      <c r="C16" s="305"/>
-      <c r="D16" s="277"/>
-      <c r="E16" s="278"/>
-      <c r="F16" s="278"/>
+      <c r="B16" s="291"/>
+      <c r="C16" s="291"/>
+      <c r="D16" s="279"/>
+      <c r="E16" s="280"/>
+      <c r="F16" s="280"/>
     </row>
     <row r="17" spans="1:12" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="241" t="s">
@@ -3035,19 +3035,19 @@
       <c r="F19" s="18"/>
     </row>
     <row r="20" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="287"/>
-      <c r="B20" s="288"/>
-      <c r="C20" s="288"/>
+      <c r="A20" s="283"/>
+      <c r="B20" s="284"/>
+      <c r="C20" s="284"/>
       <c r="D20" s="207"/>
       <c r="E20" s="51"/>
       <c r="F20" s="201"/>
     </row>
     <row r="21" spans="1:12" ht="24.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="304" t="s">
+      <c r="A21" s="286" t="s">
         <v>298</v>
       </c>
-      <c r="B21" s="304"/>
-      <c r="C21" s="304"/>
+      <c r="B21" s="286"/>
+      <c r="C21" s="286"/>
       <c r="D21" s="207"/>
       <c r="E21" s="18"/>
       <c r="F21" s="18"/>
@@ -3071,9 +3071,9 @@
       <c r="F23" s="203"/>
     </row>
     <row r="24" spans="1:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="287"/>
-      <c r="B24" s="288"/>
-      <c r="C24" s="289"/>
+      <c r="A24" s="283"/>
+      <c r="B24" s="284"/>
+      <c r="C24" s="285"/>
       <c r="D24" s="207"/>
       <c r="E24" s="204"/>
       <c r="F24" s="203"/>
@@ -3081,11 +3081,11 @@
       <c r="L24" s="18"/>
     </row>
     <row r="25" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="283" t="s">
+      <c r="A25" s="287" t="s">
         <v>297</v>
       </c>
-      <c r="B25" s="284"/>
-      <c r="C25" s="284"/>
+      <c r="B25" s="288"/>
+      <c r="C25" s="288"/>
       <c r="D25" s="223"/>
       <c r="E25" s="224"/>
       <c r="F25" s="224"/>
@@ -3121,19 +3121,19 @@
       <c r="F27" s="227"/>
     </row>
     <row r="28" spans="1:12" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="287"/>
-      <c r="B28" s="288"/>
-      <c r="C28" s="288"/>
+      <c r="A28" s="283"/>
+      <c r="B28" s="284"/>
+      <c r="C28" s="284"/>
       <c r="D28" s="207"/>
       <c r="E28" s="18"/>
       <c r="F28" s="18"/>
     </row>
     <row r="29" spans="1:12" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="285" t="s">
+      <c r="A29" s="289" t="s">
         <v>300</v>
       </c>
-      <c r="B29" s="286"/>
-      <c r="C29" s="286"/>
+      <c r="B29" s="290"/>
+      <c r="C29" s="290"/>
       <c r="D29" s="205"/>
       <c r="E29" s="37"/>
       <c r="F29" s="37"/>
@@ -3157,19 +3157,19 @@
       <c r="F31" s="37"/>
     </row>
     <row r="32" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="288"/>
-      <c r="B32" s="288"/>
-      <c r="C32" s="289"/>
+      <c r="A32" s="284"/>
+      <c r="B32" s="284"/>
+      <c r="C32" s="285"/>
       <c r="D32" s="207"/>
       <c r="E32" s="18"/>
       <c r="F32" s="18"/>
     </row>
     <row r="33" spans="1:6" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="285" t="s">
+      <c r="A33" s="289" t="s">
         <v>45</v>
       </c>
-      <c r="B33" s="286"/>
-      <c r="C33" s="286"/>
+      <c r="B33" s="290"/>
+      <c r="C33" s="290"/>
       <c r="D33" s="205"/>
       <c r="E33" s="37"/>
       <c r="F33" s="37"/>
@@ -3185,18 +3185,18 @@
       <c r="F34" s="37"/>
     </row>
     <row r="35" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="290"/>
-      <c r="B35" s="291"/>
-      <c r="C35" s="292"/>
+      <c r="A35" s="300"/>
+      <c r="B35" s="301"/>
+      <c r="C35" s="302"/>
       <c r="D35" s="208"/>
       <c r="F35" s="209"/>
     </row>
     <row r="36" spans="1:6" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="302" t="s">
+      <c r="A36" s="281" t="s">
         <v>301</v>
       </c>
-      <c r="B36" s="303"/>
-      <c r="C36" s="303"/>
+      <c r="B36" s="282"/>
+      <c r="C36" s="282"/>
       <c r="D36" s="208"/>
     </row>
     <row r="37" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -3208,26 +3208,26 @@
       <c r="D37" s="208"/>
     </row>
     <row r="38" spans="1:6" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="293"/>
-      <c r="B38" s="294"/>
-      <c r="C38" s="295"/>
+      <c r="A38" s="303"/>
+      <c r="B38" s="304"/>
+      <c r="C38" s="305"/>
       <c r="D38" s="208"/>
       <c r="F38" s="209"/>
     </row>
     <row r="39" spans="1:6" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="302" t="s">
+      <c r="A39" s="281" t="s">
         <v>40</v>
       </c>
-      <c r="B39" s="303"/>
-      <c r="C39" s="303"/>
+      <c r="B39" s="282"/>
+      <c r="C39" s="282"/>
       <c r="D39" s="208"/>
       <c r="F39" s="209"/>
     </row>
     <row r="40" spans="1:6" s="216" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="279" t="s">
+      <c r="A40" s="296" t="s">
         <v>74</v>
       </c>
-      <c r="B40" s="280"/>
+      <c r="B40" s="297"/>
       <c r="C40" s="235"/>
       <c r="D40" s="211"/>
       <c r="F40" s="212"/>
@@ -3241,10 +3241,10 @@
       <c r="D41" s="208"/>
     </row>
     <row r="42" spans="1:6" s="216" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="279" t="s">
+      <c r="A42" s="296" t="s">
         <v>75</v>
       </c>
-      <c r="B42" s="280"/>
+      <c r="B42" s="297"/>
       <c r="C42" s="236"/>
       <c r="D42" s="213"/>
       <c r="E42" s="228"/>
@@ -3261,30 +3261,30 @@
       <c r="F43" s="198"/>
     </row>
     <row r="44" spans="1:6" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="287"/>
-      <c r="B44" s="288"/>
-      <c r="C44" s="289"/>
+      <c r="A44" s="283"/>
+      <c r="B44" s="284"/>
+      <c r="C44" s="285"/>
       <c r="D44" s="207"/>
       <c r="E44" s="18"/>
       <c r="F44" s="198"/>
     </row>
     <row r="45" spans="1:6" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="281" t="s">
+      <c r="A45" s="298" t="s">
         <v>324</v>
       </c>
-      <c r="B45" s="282"/>
-      <c r="C45" s="282"/>
-      <c r="D45" s="282"/>
+      <c r="B45" s="299"/>
+      <c r="C45" s="299"/>
+      <c r="D45" s="299"/>
       <c r="E45" s="207"/>
       <c r="F45" s="198"/>
     </row>
     <row r="46" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="135"/>
-      <c r="B46" s="273" t="s">
+      <c r="B46" s="292" t="s">
         <v>317</v>
       </c>
-      <c r="C46" s="274"/>
-      <c r="D46" s="274"/>
+      <c r="C46" s="293"/>
+      <c r="D46" s="293"/>
       <c r="E46" s="208"/>
       <c r="F46"/>
     </row>
@@ -3322,11 +3322,11 @@
     </row>
     <row r="50" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="253"/>
-      <c r="B50" s="275" t="s">
+      <c r="B50" s="294" t="s">
         <v>4</v>
       </c>
-      <c r="C50" s="276"/>
-      <c r="D50" s="276"/>
+      <c r="C50" s="295"/>
+      <c r="D50" s="295"/>
       <c r="E50" s="206"/>
       <c r="F50" s="28"/>
       <c r="J50" s="202"/>
@@ -3401,6 +3401,19 @@
     </row>
   </sheetData>
   <mergeCells count="29">
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="B50:D50"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="A45:D45"/>
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="A44:C44"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="D7:F7"/>
@@ -3417,19 +3430,6 @@
     <mergeCell ref="A16:C16"/>
     <mergeCell ref="A33:C33"/>
     <mergeCell ref="A21:C21"/>
-    <mergeCell ref="B46:D46"/>
-    <mergeCell ref="B50:D50"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="A42:B42"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="A45:D45"/>
-    <mergeCell ref="A25:C25"/>
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="A38:C38"/>
-    <mergeCell ref="A44:C44"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.25" header="0.3" footer="0.3"/>
   <pageSetup scale="69" fitToHeight="0" orientation="portrait" r:id="rId1"/>
@@ -6323,14 +6323,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="23.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="325" t="s">
+      <c r="A1" s="314" t="s">
         <v>207</v>
       </c>
-      <c r="B1" s="325"/>
-      <c r="C1" s="325"/>
-      <c r="D1" s="325"/>
-      <c r="E1" s="325"/>
-      <c r="F1" s="325"/>
+      <c r="B1" s="314"/>
+      <c r="C1" s="314"/>
+      <c r="D1" s="314"/>
+      <c r="E1" s="314"/>
+      <c r="F1" s="314"/>
     </row>
     <row r="2" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2"/>
@@ -6746,12 +6746,12 @@
       <c r="G25" s="1"/>
     </row>
     <row r="26" spans="1:7" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="326"/>
-      <c r="B26" s="327"/>
-      <c r="C26" s="327"/>
-      <c r="D26" s="327"/>
-      <c r="E26" s="327"/>
-      <c r="F26" s="327"/>
+      <c r="A26" s="315"/>
+      <c r="B26" s="316"/>
+      <c r="C26" s="316"/>
+      <c r="D26" s="316"/>
+      <c r="E26" s="316"/>
+      <c r="F26" s="316"/>
       <c r="G26" s="1"/>
     </row>
     <row r="27" spans="1:7" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -6834,23 +6834,23 @@
       <c r="G32" s="1"/>
     </row>
     <row r="33" spans="1:7" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="328"/>
-      <c r="B33" s="323"/>
-      <c r="C33" s="323"/>
-      <c r="D33" s="323"/>
-      <c r="E33" s="323"/>
-      <c r="F33" s="324"/>
+      <c r="A33" s="317"/>
+      <c r="B33" s="312"/>
+      <c r="C33" s="312"/>
+      <c r="D33" s="312"/>
+      <c r="E33" s="312"/>
+      <c r="F33" s="313"/>
       <c r="G33" s="1"/>
     </row>
     <row r="34" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="109" t="s">
         <v>36</v>
       </c>
-      <c r="B34" s="323"/>
-      <c r="C34" s="323"/>
-      <c r="D34" s="323"/>
-      <c r="E34" s="323"/>
-      <c r="F34" s="324"/>
+      <c r="B34" s="312"/>
+      <c r="C34" s="312"/>
+      <c r="D34" s="312"/>
+      <c r="E34" s="312"/>
+      <c r="F34" s="313"/>
       <c r="G34" s="1"/>
     </row>
     <row r="35" spans="1:7" s="106" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.35">
@@ -6889,12 +6889,12 @@
       <c r="G37" s="1"/>
     </row>
     <row r="38" spans="1:7" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="312"/>
-      <c r="B38" s="313"/>
-      <c r="C38" s="313"/>
-      <c r="D38" s="313"/>
-      <c r="E38" s="313"/>
-      <c r="F38" s="314"/>
+      <c r="A38" s="318"/>
+      <c r="B38" s="319"/>
+      <c r="C38" s="319"/>
+      <c r="D38" s="319"/>
+      <c r="E38" s="319"/>
+      <c r="F38" s="320"/>
       <c r="G38" s="1"/>
     </row>
     <row r="39" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
@@ -7059,12 +7059,12 @@
       <c r="G49" s="1"/>
     </row>
     <row r="50" spans="1:7" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="312"/>
-      <c r="B50" s="313"/>
-      <c r="C50" s="313"/>
-      <c r="D50" s="313"/>
-      <c r="E50" s="313"/>
-      <c r="F50" s="314"/>
+      <c r="A50" s="318"/>
+      <c r="B50" s="319"/>
+      <c r="C50" s="319"/>
+      <c r="D50" s="319"/>
+      <c r="E50" s="319"/>
+      <c r="F50" s="320"/>
       <c r="G50" s="1"/>
     </row>
     <row r="51" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
@@ -7255,14 +7255,14 @@
       <c r="G71" s="1"/>
     </row>
     <row r="72" spans="1:15" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A72" s="315" t="s">
+      <c r="A72" s="321" t="s">
         <v>75</v>
       </c>
-      <c r="B72" s="316"/>
-      <c r="C72" s="316"/>
-      <c r="D72" s="316"/>
-      <c r="E72" s="316"/>
-      <c r="F72" s="317"/>
+      <c r="B72" s="322"/>
+      <c r="C72" s="322"/>
+      <c r="D72" s="322"/>
+      <c r="E72" s="322"/>
+      <c r="F72" s="323"/>
       <c r="G72" s="1"/>
     </row>
     <row r="73" spans="1:15" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -7332,21 +7332,21 @@
       <c r="G77" s="1"/>
     </row>
     <row r="78" spans="1:15" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A78" s="318" t="s">
+      <c r="A78" s="324" t="s">
         <v>68</v>
       </c>
-      <c r="B78" s="320" t="s">
+      <c r="B78" s="326" t="s">
         <v>3</v>
       </c>
-      <c r="C78" s="320"/>
-      <c r="E78" s="321" t="s">
+      <c r="C78" s="326"/>
+      <c r="E78" s="327" t="s">
         <v>4</v>
       </c>
-      <c r="F78" s="322"/>
+      <c r="F78" s="328"/>
       <c r="G78" s="1"/>
     </row>
     <row r="79" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A79" s="319"/>
+      <c r="A79" s="325"/>
       <c r="B79" s="52" t="s">
         <v>52</v>
       </c>
@@ -7578,16 +7578,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A50:F50"/>
+    <mergeCell ref="A72:F72"/>
+    <mergeCell ref="A78:A79"/>
+    <mergeCell ref="B78:C78"/>
+    <mergeCell ref="E78:F78"/>
     <mergeCell ref="B34:F34"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A26:F26"/>
     <mergeCell ref="A33:F33"/>
     <mergeCell ref="A38:F38"/>
-    <mergeCell ref="A50:F50"/>
-    <mergeCell ref="A72:F72"/>
-    <mergeCell ref="A78:A79"/>
-    <mergeCell ref="B78:C78"/>
-    <mergeCell ref="E78:F78"/>
   </mergeCells>
   <printOptions horizontalCentered="1" gridLines="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7618,14 +7618,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="23.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="325" t="s">
+      <c r="A1" s="314" t="s">
         <v>185</v>
       </c>
-      <c r="B1" s="325"/>
-      <c r="C1" s="325"/>
-      <c r="D1" s="325"/>
-      <c r="E1" s="325"/>
-      <c r="F1" s="325"/>
+      <c r="B1" s="314"/>
+      <c r="C1" s="314"/>
+      <c r="D1" s="314"/>
+      <c r="E1" s="314"/>
+      <c r="F1" s="314"/>
     </row>
     <row r="2" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2"/>
@@ -7896,10 +7896,10 @@
         <v>33</v>
       </c>
       <c r="B18" s="329"/>
-      <c r="C18" s="321"/>
-      <c r="D18" s="321"/>
-      <c r="E18" s="321"/>
-      <c r="F18" s="322"/>
+      <c r="C18" s="327"/>
+      <c r="D18" s="327"/>
+      <c r="E18" s="327"/>
+      <c r="F18" s="328"/>
       <c r="G18" s="1"/>
     </row>
     <row r="19" spans="1:7" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -7986,12 +7986,12 @@
       <c r="G22" s="1"/>
     </row>
     <row r="23" spans="1:7" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="326"/>
-      <c r="B23" s="327"/>
-      <c r="C23" s="327"/>
-      <c r="D23" s="327"/>
-      <c r="E23" s="327"/>
-      <c r="F23" s="327"/>
+      <c r="A23" s="315"/>
+      <c r="B23" s="316"/>
+      <c r="C23" s="316"/>
+      <c r="D23" s="316"/>
+      <c r="E23" s="316"/>
+      <c r="F23" s="316"/>
       <c r="G23" s="1"/>
     </row>
     <row r="24" spans="1:7" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -8019,10 +8019,10 @@
         <v>22</v>
       </c>
       <c r="B25" s="329"/>
-      <c r="C25" s="321"/>
-      <c r="D25" s="321"/>
-      <c r="E25" s="321"/>
-      <c r="F25" s="322"/>
+      <c r="C25" s="327"/>
+      <c r="D25" s="327"/>
+      <c r="E25" s="327"/>
+      <c r="F25" s="328"/>
       <c r="G25" s="1"/>
     </row>
     <row r="26" spans="1:7" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -8126,23 +8126,23 @@
       <c r="G30" s="1"/>
     </row>
     <row r="31" spans="1:7" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="328"/>
-      <c r="B31" s="323"/>
-      <c r="C31" s="323"/>
-      <c r="D31" s="323"/>
-      <c r="E31" s="323"/>
-      <c r="F31" s="324"/>
+      <c r="A31" s="317"/>
+      <c r="B31" s="312"/>
+      <c r="C31" s="312"/>
+      <c r="D31" s="312"/>
+      <c r="E31" s="312"/>
+      <c r="F31" s="313"/>
       <c r="G31" s="1"/>
     </row>
     <row r="32" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="B32" s="323"/>
-      <c r="C32" s="323"/>
-      <c r="D32" s="323"/>
-      <c r="E32" s="323"/>
-      <c r="F32" s="324"/>
+      <c r="B32" s="312"/>
+      <c r="C32" s="312"/>
+      <c r="D32" s="312"/>
+      <c r="E32" s="312"/>
+      <c r="F32" s="313"/>
       <c r="G32" s="1"/>
     </row>
     <row r="33" spans="1:7" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -8191,12 +8191,12 @@
       <c r="G35" s="1"/>
     </row>
     <row r="36" spans="1:7" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="312"/>
-      <c r="B36" s="313"/>
-      <c r="C36" s="313"/>
-      <c r="D36" s="313"/>
-      <c r="E36" s="313"/>
-      <c r="F36" s="314"/>
+      <c r="A36" s="318"/>
+      <c r="B36" s="319"/>
+      <c r="C36" s="319"/>
+      <c r="D36" s="319"/>
+      <c r="E36" s="319"/>
+      <c r="F36" s="320"/>
       <c r="G36" s="1"/>
     </row>
     <row r="37" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
@@ -8361,12 +8361,12 @@
       <c r="G47" s="1"/>
     </row>
     <row r="48" spans="1:7" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="312"/>
-      <c r="B48" s="313"/>
-      <c r="C48" s="313"/>
-      <c r="D48" s="313"/>
-      <c r="E48" s="313"/>
-      <c r="F48" s="314"/>
+      <c r="A48" s="318"/>
+      <c r="B48" s="319"/>
+      <c r="C48" s="319"/>
+      <c r="D48" s="319"/>
+      <c r="E48" s="319"/>
+      <c r="F48" s="320"/>
       <c r="G48" s="1"/>
     </row>
     <row r="49" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.35">
@@ -8572,14 +8572,14 @@
       <c r="G69" s="1"/>
     </row>
     <row r="70" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A70" s="315" t="s">
+      <c r="A70" s="321" t="s">
         <v>75</v>
       </c>
-      <c r="B70" s="316"/>
-      <c r="C70" s="316"/>
-      <c r="D70" s="316"/>
-      <c r="E70" s="316"/>
-      <c r="F70" s="317"/>
+      <c r="B70" s="322"/>
+      <c r="C70" s="322"/>
+      <c r="D70" s="322"/>
+      <c r="E70" s="322"/>
+      <c r="F70" s="323"/>
       <c r="G70" s="1"/>
     </row>
     <row r="71" spans="1:7" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -8655,21 +8655,21 @@
       <c r="G76" s="1"/>
     </row>
     <row r="77" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A77" s="318" t="s">
+      <c r="A77" s="324" t="s">
         <v>68</v>
       </c>
-      <c r="B77" s="320" t="s">
+      <c r="B77" s="326" t="s">
         <v>3</v>
       </c>
-      <c r="C77" s="320"/>
-      <c r="E77" s="321" t="s">
+      <c r="C77" s="326"/>
+      <c r="E77" s="327" t="s">
         <v>4</v>
       </c>
-      <c r="F77" s="322"/>
+      <c r="F77" s="328"/>
       <c r="G77" s="1"/>
     </row>
     <row r="78" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A78" s="319"/>
+      <c r="A78" s="325"/>
       <c r="B78" s="52" t="s">
         <v>52</v>
       </c>
@@ -8978,18 +8978,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="B25:F25"/>
+    <mergeCell ref="A31:F31"/>
     <mergeCell ref="A36:F36"/>
     <mergeCell ref="A48:F48"/>
     <mergeCell ref="A70:F70"/>
     <mergeCell ref="A77:A78"/>
     <mergeCell ref="B77:C77"/>
     <mergeCell ref="E77:F77"/>
-    <mergeCell ref="B32:F32"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B18:F18"/>
-    <mergeCell ref="A23:F23"/>
-    <mergeCell ref="B25:F25"/>
-    <mergeCell ref="A31:F31"/>
   </mergeCells>
   <printOptions horizontalCentered="1" gridLines="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9017,14 +9017,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="23.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="325" t="s">
+      <c r="A1" s="314" t="s">
         <v>79</v>
       </c>
-      <c r="B1" s="325"/>
-      <c r="C1" s="325"/>
-      <c r="D1" s="325"/>
-      <c r="E1" s="325"/>
-      <c r="F1" s="325"/>
+      <c r="B1" s="314"/>
+      <c r="C1" s="314"/>
+      <c r="D1" s="314"/>
+      <c r="E1" s="314"/>
+      <c r="F1" s="314"/>
     </row>
     <row r="2" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2"/>
@@ -9272,10 +9272,10 @@
         <v>33</v>
       </c>
       <c r="B16" s="329"/>
-      <c r="C16" s="321"/>
-      <c r="D16" s="321"/>
-      <c r="E16" s="321"/>
-      <c r="F16" s="322"/>
+      <c r="C16" s="327"/>
+      <c r="D16" s="327"/>
+      <c r="E16" s="327"/>
+      <c r="F16" s="328"/>
       <c r="G16" s="1"/>
     </row>
     <row r="17" spans="1:7" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -9319,12 +9319,12 @@
       <c r="G20" s="1"/>
     </row>
     <row r="21" spans="1:7" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="326"/>
-      <c r="B21" s="327"/>
-      <c r="C21" s="327"/>
-      <c r="D21" s="327"/>
-      <c r="E21" s="327"/>
-      <c r="F21" s="327"/>
+      <c r="A21" s="315"/>
+      <c r="B21" s="316"/>
+      <c r="C21" s="316"/>
+      <c r="D21" s="316"/>
+      <c r="E21" s="316"/>
+      <c r="F21" s="316"/>
       <c r="G21" s="1"/>
     </row>
     <row r="22" spans="1:7" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -9355,10 +9355,10 @@
         <v>22</v>
       </c>
       <c r="B23" s="329"/>
-      <c r="C23" s="321"/>
-      <c r="D23" s="321"/>
-      <c r="E23" s="321"/>
-      <c r="F23" s="322"/>
+      <c r="C23" s="327"/>
+      <c r="D23" s="327"/>
+      <c r="E23" s="327"/>
+      <c r="F23" s="328"/>
       <c r="G23" s="1"/>
     </row>
     <row r="24" spans="1:7" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -9445,23 +9445,23 @@
       <c r="G28" s="1"/>
     </row>
     <row r="29" spans="1:7" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="328"/>
-      <c r="B29" s="323"/>
-      <c r="C29" s="323"/>
-      <c r="D29" s="323"/>
-      <c r="E29" s="323"/>
-      <c r="F29" s="324"/>
+      <c r="A29" s="317"/>
+      <c r="B29" s="312"/>
+      <c r="C29" s="312"/>
+      <c r="D29" s="312"/>
+      <c r="E29" s="312"/>
+      <c r="F29" s="313"/>
       <c r="G29" s="1"/>
     </row>
     <row r="30" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="B30" s="323"/>
-      <c r="C30" s="323"/>
-      <c r="D30" s="323"/>
-      <c r="E30" s="323"/>
-      <c r="F30" s="324"/>
+      <c r="B30" s="312"/>
+      <c r="C30" s="312"/>
+      <c r="D30" s="312"/>
+      <c r="E30" s="312"/>
+      <c r="F30" s="313"/>
       <c r="G30" s="1"/>
     </row>
     <row r="31" spans="1:7" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -9498,12 +9498,12 @@
       <c r="G33" s="1"/>
     </row>
     <row r="34" spans="1:7" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="312"/>
-      <c r="B34" s="313"/>
-      <c r="C34" s="313"/>
-      <c r="D34" s="313"/>
-      <c r="E34" s="313"/>
-      <c r="F34" s="314"/>
+      <c r="A34" s="318"/>
+      <c r="B34" s="319"/>
+      <c r="C34" s="319"/>
+      <c r="D34" s="319"/>
+      <c r="E34" s="319"/>
+      <c r="F34" s="320"/>
       <c r="G34" s="1"/>
     </row>
     <row r="35" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
@@ -9608,12 +9608,12 @@
       <c r="G41" s="1"/>
     </row>
     <row r="42" spans="1:7" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="312"/>
-      <c r="B42" s="313"/>
-      <c r="C42" s="313"/>
-      <c r="D42" s="313"/>
-      <c r="E42" s="313"/>
-      <c r="F42" s="314"/>
+      <c r="A42" s="318"/>
+      <c r="B42" s="319"/>
+      <c r="C42" s="319"/>
+      <c r="D42" s="319"/>
+      <c r="E42" s="319"/>
+      <c r="F42" s="320"/>
       <c r="G42" s="1"/>
     </row>
     <row r="43" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
@@ -9814,14 +9814,14 @@
       <c r="G63" s="1"/>
     </row>
     <row r="64" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A64" s="315" t="s">
+      <c r="A64" s="321" t="s">
         <v>75</v>
       </c>
-      <c r="B64" s="316"/>
-      <c r="C64" s="316"/>
-      <c r="D64" s="316"/>
-      <c r="E64" s="316"/>
-      <c r="F64" s="317"/>
+      <c r="B64" s="322"/>
+      <c r="C64" s="322"/>
+      <c r="D64" s="322"/>
+      <c r="E64" s="322"/>
+      <c r="F64" s="323"/>
       <c r="G64" s="1"/>
     </row>
     <row r="65" spans="1:7" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -9897,21 +9897,21 @@
       <c r="G70" s="1"/>
     </row>
     <row r="71" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A71" s="318" t="s">
+      <c r="A71" s="324" t="s">
         <v>68</v>
       </c>
-      <c r="B71" s="320" t="s">
+      <c r="B71" s="326" t="s">
         <v>3</v>
       </c>
-      <c r="C71" s="320"/>
-      <c r="E71" s="321" t="s">
+      <c r="C71" s="326"/>
+      <c r="E71" s="327" t="s">
         <v>4</v>
       </c>
-      <c r="F71" s="322"/>
+      <c r="F71" s="328"/>
       <c r="G71" s="1"/>
     </row>
     <row r="72" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A72" s="319"/>
+      <c r="A72" s="325"/>
       <c r="B72" s="52" t="s">
         <v>52</v>
       </c>
@@ -10688,11 +10688,11 @@
       <c r="F30" s="1"/>
     </row>
     <row r="31" spans="1:6" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="312"/>
-      <c r="B31" s="313"/>
-      <c r="C31" s="313"/>
-      <c r="D31" s="313"/>
-      <c r="E31" s="314"/>
+      <c r="A31" s="318"/>
+      <c r="B31" s="319"/>
+      <c r="C31" s="319"/>
+      <c r="D31" s="319"/>
+      <c r="E31" s="320"/>
       <c r="F31" s="1"/>
     </row>
     <row r="32" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.35">
@@ -10786,11 +10786,11 @@
       <c r="F38" s="1"/>
     </row>
     <row r="39" spans="1:6" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="312"/>
-      <c r="B39" s="313"/>
-      <c r="C39" s="313"/>
-      <c r="D39" s="313"/>
-      <c r="E39" s="314"/>
+      <c r="A39" s="318"/>
+      <c r="B39" s="319"/>
+      <c r="C39" s="319"/>
+      <c r="D39" s="319"/>
+      <c r="E39" s="320"/>
       <c r="F39" s="1"/>
     </row>
     <row r="40" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.35">
@@ -10996,13 +10996,13 @@
       <c r="F61" s="1"/>
     </row>
     <row r="62" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A62" s="315" t="s">
+      <c r="A62" s="321" t="s">
         <v>124</v>
       </c>
-      <c r="B62" s="316"/>
-      <c r="C62" s="316"/>
-      <c r="D62" s="316"/>
-      <c r="E62" s="317"/>
+      <c r="B62" s="322"/>
+      <c r="C62" s="322"/>
+      <c r="D62" s="322"/>
+      <c r="E62" s="323"/>
       <c r="F62" s="1"/>
     </row>
     <row r="63" spans="1:6" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -11080,13 +11080,13 @@
       <c r="F68" s="1"/>
     </row>
     <row r="69" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A69" s="318" t="s">
+      <c r="A69" s="324" t="s">
         <v>126</v>
       </c>
-      <c r="B69" s="320" t="s">
+      <c r="B69" s="326" t="s">
         <v>3</v>
       </c>
-      <c r="C69" s="320"/>
+      <c r="C69" s="326"/>
       <c r="D69" s="33" t="s">
         <v>4</v>
       </c>
@@ -11094,7 +11094,7 @@
       <c r="F69" s="1"/>
     </row>
     <row r="70" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A70" s="319"/>
+      <c r="A70" s="325"/>
       <c r="B70" s="52" t="s">
         <v>52</v>
       </c>
@@ -11371,34 +11371,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="27" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="334">
+      <c r="A1" s="333">
         <v>2017</v>
       </c>
-      <c r="B1" s="335"/>
-      <c r="C1" s="335"/>
-      <c r="D1" s="335"/>
-      <c r="E1" s="335"/>
-      <c r="F1" s="335"/>
-      <c r="G1" s="335"/>
-      <c r="H1" s="335"/>
-      <c r="I1" s="335"/>
-      <c r="J1" s="335"/>
-      <c r="K1" s="336"/>
+      <c r="B1" s="334"/>
+      <c r="C1" s="334"/>
+      <c r="D1" s="334"/>
+      <c r="E1" s="334"/>
+      <c r="F1" s="334"/>
+      <c r="G1" s="334"/>
+      <c r="H1" s="334"/>
+      <c r="I1" s="334"/>
+      <c r="J1" s="334"/>
+      <c r="K1" s="335"/>
     </row>
     <row r="2" spans="1:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="337" t="s">
+      <c r="A2" s="336" t="s">
         <v>133</v>
       </c>
-      <c r="B2" s="337"/>
-      <c r="C2" s="337"/>
-      <c r="D2" s="337"/>
-      <c r="E2" s="337"/>
-      <c r="F2" s="337"/>
-      <c r="G2" s="337"/>
-      <c r="H2" s="337"/>
-      <c r="I2" s="337"/>
-      <c r="J2" s="337"/>
-      <c r="K2" s="337"/>
+      <c r="B2" s="336"/>
+      <c r="C2" s="336"/>
+      <c r="D2" s="336"/>
+      <c r="E2" s="336"/>
+      <c r="F2" s="336"/>
+      <c r="G2" s="336"/>
+      <c r="H2" s="336"/>
+      <c r="I2" s="336"/>
+      <c r="J2" s="336"/>
+      <c r="K2" s="336"/>
       <c r="L2" s="66"/>
       <c r="M2" s="66"/>
       <c r="N2" s="66"/>
@@ -11422,10 +11422,10 @@
       <c r="E6" s="68">
         <v>0.13420000000000001</v>
       </c>
-      <c r="F6" s="338" t="s">
+      <c r="F6" s="337" t="s">
         <v>136</v>
       </c>
-      <c r="G6" s="338"/>
+      <c r="G6" s="337"/>
       <c r="L6" s="69"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
@@ -11438,10 +11438,10 @@
       <c r="E7" s="70">
         <v>0.37</v>
       </c>
-      <c r="F7" s="338" t="s">
+      <c r="F7" s="337" t="s">
         <v>138</v>
       </c>
-      <c r="G7" s="338"/>
+      <c r="G7" s="337"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="E8" s="70"/>
@@ -12007,10 +12007,10 @@
       <c r="K52" s="80"/>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A53" s="333" t="s">
+      <c r="A53" s="338" t="s">
         <v>183</v>
       </c>
-      <c r="B53" s="333"/>
+      <c r="B53" s="338"/>
       <c r="C53" s="82">
         <v>16.73</v>
       </c>
@@ -12115,12 +12115,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="A21:B21"/>
     <mergeCell ref="A50:B50"/>
     <mergeCell ref="A53:B53"/>
     <mergeCell ref="A40:D40"/>
@@ -12129,6 +12123,12 @@
     <mergeCell ref="A45:B45"/>
     <mergeCell ref="A46:B46"/>
     <mergeCell ref="A47:B47"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="A21:B21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
show route success as %
</commit_message>
<xml_diff>
--- a/web/flask/static/annual_report_template.xlsx
+++ b/web/flask/static/annual_report_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\apps\climberdb\git\web\flask\static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D332130-0012-4C53-82F4-290A1EC0F289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A899115-AB0F-403D-9E2A-1E6683002862}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2325,7 +2325,6 @@
     <xf numFmtId="0" fontId="9" fillId="7" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -2338,10 +2337,78 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2360,87 +2427,18 @@
     <xf numFmtId="0" fontId="19" fillId="8" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="8" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="8" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="21" fillId="9" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="21" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2459,6 +2457,39 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2477,39 +2508,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2522,6 +2520,9 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2537,8 +2538,11 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2843,24 +2847,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="61.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="273" t="s">
+      <c r="A1" s="294" t="s">
         <v>325</v>
       </c>
-      <c r="B1" s="274"/>
-      <c r="C1" s="274"/>
-      <c r="D1" s="274"/>
-      <c r="E1" s="274"/>
-      <c r="F1" s="275"/>
+      <c r="B1" s="295"/>
+      <c r="C1" s="295"/>
+      <c r="D1" s="295"/>
+      <c r="E1" s="295"/>
+      <c r="F1" s="296"/>
     </row>
     <row r="2" spans="1:6" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="276" t="s">
+      <c r="A2" s="297" t="s">
         <v>290</v>
       </c>
-      <c r="B2" s="277"/>
-      <c r="C2" s="277"/>
-      <c r="D2" s="277"/>
-      <c r="E2" s="277"/>
-      <c r="F2" s="278"/>
+      <c r="B2" s="298"/>
+      <c r="C2" s="298"/>
+      <c r="D2" s="298"/>
+      <c r="E2" s="298"/>
+      <c r="F2" s="299"/>
     </row>
     <row r="3" spans="1:6" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="229" t="s">
@@ -2881,32 +2885,32 @@
       <c r="F4" s="261"/>
     </row>
     <row r="5" spans="1:6" ht="24.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="283"/>
-      <c r="B5" s="284"/>
-      <c r="C5" s="284"/>
+      <c r="A5" s="285"/>
+      <c r="B5" s="286"/>
+      <c r="C5" s="286"/>
       <c r="D5" s="217"/>
       <c r="E5" s="218"/>
       <c r="F5" s="219"/>
     </row>
     <row r="6" spans="1:6" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="289" t="s">
+      <c r="A6" s="283" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="290"/>
-      <c r="C6" s="290"/>
+      <c r="B6" s="284"/>
+      <c r="C6" s="284"/>
       <c r="D6" s="220"/>
       <c r="E6" s="221"/>
       <c r="F6" s="221"/>
     </row>
     <row r="7" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="287" t="s">
+      <c r="A7" s="281" t="s">
         <v>291</v>
       </c>
-      <c r="B7" s="288"/>
-      <c r="C7" s="288"/>
-      <c r="D7" s="279"/>
-      <c r="E7" s="280"/>
-      <c r="F7" s="280"/>
+      <c r="B7" s="282"/>
+      <c r="C7" s="282"/>
+      <c r="D7" s="275"/>
+      <c r="E7" s="276"/>
+      <c r="F7" s="276"/>
     </row>
     <row r="8" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="241" t="s">
@@ -2945,19 +2949,19 @@
       <c r="F10" s="18"/>
     </row>
     <row r="11" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="283"/>
-      <c r="B11" s="284"/>
-      <c r="C11" s="284"/>
+      <c r="A11" s="285"/>
+      <c r="B11" s="286"/>
+      <c r="C11" s="286"/>
       <c r="D11" s="210"/>
       <c r="E11" s="18"/>
       <c r="F11" s="18"/>
     </row>
     <row r="12" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="286" t="s">
+      <c r="A12" s="302" t="s">
         <v>231</v>
       </c>
-      <c r="B12" s="286"/>
-      <c r="C12" s="286"/>
+      <c r="B12" s="302"/>
+      <c r="C12" s="302"/>
       <c r="D12" s="210"/>
       <c r="E12" s="18"/>
       <c r="F12" s="18"/>
@@ -2975,28 +2979,28 @@
     <row r="14" spans="1:6" ht="27" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="257"/>
       <c r="B14" s="242"/>
-      <c r="C14" s="267"/>
+      <c r="C14" s="266"/>
       <c r="D14" s="208"/>
       <c r="E14" s="199"/>
       <c r="F14" s="51"/>
     </row>
     <row r="15" spans="1:6" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="283"/>
-      <c r="B15" s="284"/>
-      <c r="C15" s="284"/>
+      <c r="A15" s="285"/>
+      <c r="B15" s="286"/>
+      <c r="C15" s="286"/>
       <c r="D15" s="223"/>
       <c r="E15" s="224"/>
       <c r="F15" s="224"/>
     </row>
     <row r="16" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="287" t="s">
+      <c r="A16" s="281" t="s">
         <v>296</v>
       </c>
-      <c r="B16" s="291"/>
-      <c r="C16" s="291"/>
-      <c r="D16" s="279"/>
-      <c r="E16" s="280"/>
-      <c r="F16" s="280"/>
+      <c r="B16" s="303"/>
+      <c r="C16" s="303"/>
+      <c r="D16" s="275"/>
+      <c r="E16" s="276"/>
+      <c r="F16" s="276"/>
     </row>
     <row r="17" spans="1:12" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="241" t="s">
@@ -3035,19 +3039,19 @@
       <c r="F19" s="18"/>
     </row>
     <row r="20" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="283"/>
-      <c r="B20" s="284"/>
-      <c r="C20" s="284"/>
+      <c r="A20" s="285"/>
+      <c r="B20" s="286"/>
+      <c r="C20" s="286"/>
       <c r="D20" s="207"/>
       <c r="E20" s="51"/>
       <c r="F20" s="201"/>
     </row>
     <row r="21" spans="1:12" ht="24.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="286" t="s">
+      <c r="A21" s="302" t="s">
         <v>298</v>
       </c>
-      <c r="B21" s="286"/>
-      <c r="C21" s="286"/>
+      <c r="B21" s="302"/>
+      <c r="C21" s="302"/>
       <c r="D21" s="207"/>
       <c r="E21" s="18"/>
       <c r="F21" s="18"/>
@@ -3071,9 +3075,9 @@
       <c r="F23" s="203"/>
     </row>
     <row r="24" spans="1:12" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="283"/>
-      <c r="B24" s="284"/>
-      <c r="C24" s="285"/>
+      <c r="A24" s="285"/>
+      <c r="B24" s="286"/>
+      <c r="C24" s="287"/>
       <c r="D24" s="207"/>
       <c r="E24" s="204"/>
       <c r="F24" s="203"/>
@@ -3081,11 +3085,11 @@
       <c r="L24" s="18"/>
     </row>
     <row r="25" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="287" t="s">
+      <c r="A25" s="281" t="s">
         <v>297</v>
       </c>
-      <c r="B25" s="288"/>
-      <c r="C25" s="288"/>
+      <c r="B25" s="282"/>
+      <c r="C25" s="282"/>
       <c r="D25" s="223"/>
       <c r="E25" s="224"/>
       <c r="F25" s="224"/>
@@ -3121,19 +3125,19 @@
       <c r="F27" s="227"/>
     </row>
     <row r="28" spans="1:12" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="283"/>
-      <c r="B28" s="284"/>
-      <c r="C28" s="284"/>
+      <c r="A28" s="285"/>
+      <c r="B28" s="286"/>
+      <c r="C28" s="286"/>
       <c r="D28" s="207"/>
       <c r="E28" s="18"/>
       <c r="F28" s="18"/>
     </row>
     <row r="29" spans="1:12" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="289" t="s">
+      <c r="A29" s="283" t="s">
         <v>300</v>
       </c>
-      <c r="B29" s="290"/>
-      <c r="C29" s="290"/>
+      <c r="B29" s="284"/>
+      <c r="C29" s="284"/>
       <c r="D29" s="205"/>
       <c r="E29" s="37"/>
       <c r="F29" s="37"/>
@@ -3157,19 +3161,19 @@
       <c r="F31" s="37"/>
     </row>
     <row r="32" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="284"/>
-      <c r="B32" s="284"/>
-      <c r="C32" s="285"/>
+      <c r="A32" s="286"/>
+      <c r="B32" s="286"/>
+      <c r="C32" s="287"/>
       <c r="D32" s="207"/>
       <c r="E32" s="18"/>
       <c r="F32" s="18"/>
     </row>
     <row r="33" spans="1:6" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="289" t="s">
+      <c r="A33" s="283" t="s">
         <v>45</v>
       </c>
-      <c r="B33" s="290"/>
-      <c r="C33" s="290"/>
+      <c r="B33" s="284"/>
+      <c r="C33" s="284"/>
       <c r="D33" s="205"/>
       <c r="E33" s="37"/>
       <c r="F33" s="37"/>
@@ -3185,18 +3189,18 @@
       <c r="F34" s="37"/>
     </row>
     <row r="35" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="300"/>
-      <c r="B35" s="301"/>
-      <c r="C35" s="302"/>
+      <c r="A35" s="288"/>
+      <c r="B35" s="289"/>
+      <c r="C35" s="290"/>
       <c r="D35" s="208"/>
       <c r="F35" s="209"/>
     </row>
     <row r="36" spans="1:6" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="281" t="s">
+      <c r="A36" s="300" t="s">
         <v>301</v>
       </c>
-      <c r="B36" s="282"/>
-      <c r="C36" s="282"/>
+      <c r="B36" s="301"/>
+      <c r="C36" s="301"/>
       <c r="D36" s="208"/>
     </row>
     <row r="37" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.35">
@@ -3208,26 +3212,26 @@
       <c r="D37" s="208"/>
     </row>
     <row r="38" spans="1:6" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="303"/>
-      <c r="B38" s="304"/>
-      <c r="C38" s="305"/>
+      <c r="A38" s="291"/>
+      <c r="B38" s="292"/>
+      <c r="C38" s="293"/>
       <c r="D38" s="208"/>
       <c r="F38" s="209"/>
     </row>
     <row r="39" spans="1:6" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="281" t="s">
+      <c r="A39" s="300" t="s">
         <v>40</v>
       </c>
-      <c r="B39" s="282"/>
-      <c r="C39" s="282"/>
+      <c r="B39" s="301"/>
+      <c r="C39" s="301"/>
       <c r="D39" s="208"/>
       <c r="F39" s="209"/>
     </row>
     <row r="40" spans="1:6" s="216" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="296" t="s">
+      <c r="A40" s="277" t="s">
         <v>74</v>
       </c>
-      <c r="B40" s="297"/>
+      <c r="B40" s="278"/>
       <c r="C40" s="235"/>
       <c r="D40" s="211"/>
       <c r="F40" s="212"/>
@@ -3241,10 +3245,10 @@
       <c r="D41" s="208"/>
     </row>
     <row r="42" spans="1:6" s="216" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="296" t="s">
+      <c r="A42" s="277" t="s">
         <v>75</v>
       </c>
-      <c r="B42" s="297"/>
+      <c r="B42" s="278"/>
       <c r="C42" s="236"/>
       <c r="D42" s="213"/>
       <c r="E42" s="228"/>
@@ -3261,30 +3265,30 @@
       <c r="F43" s="198"/>
     </row>
     <row r="44" spans="1:6" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="283"/>
-      <c r="B44" s="284"/>
-      <c r="C44" s="285"/>
+      <c r="A44" s="285"/>
+      <c r="B44" s="286"/>
+      <c r="C44" s="287"/>
       <c r="D44" s="207"/>
       <c r="E44" s="18"/>
       <c r="F44" s="198"/>
     </row>
     <row r="45" spans="1:6" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="298" t="s">
+      <c r="A45" s="279" t="s">
         <v>324</v>
       </c>
-      <c r="B45" s="299"/>
-      <c r="C45" s="299"/>
-      <c r="D45" s="299"/>
+      <c r="B45" s="280"/>
+      <c r="C45" s="280"/>
+      <c r="D45" s="280"/>
       <c r="E45" s="207"/>
       <c r="F45" s="198"/>
     </row>
     <row r="46" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="135"/>
-      <c r="B46" s="292" t="s">
+      <c r="B46" s="271" t="s">
         <v>317</v>
       </c>
-      <c r="C46" s="293"/>
-      <c r="D46" s="293"/>
+      <c r="C46" s="272"/>
+      <c r="D46" s="272"/>
       <c r="E46" s="208"/>
       <c r="F46"/>
     </row>
@@ -3308,7 +3312,7 @@
       <c r="A48" s="196"/>
       <c r="B48" s="197"/>
       <c r="C48" s="249"/>
-      <c r="D48" s="266"/>
+      <c r="D48" s="337"/>
       <c r="E48" s="207"/>
       <c r="F48" s="201"/>
     </row>
@@ -3322,11 +3326,11 @@
     </row>
     <row r="50" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="253"/>
-      <c r="B50" s="294" t="s">
+      <c r="B50" s="273" t="s">
         <v>4</v>
       </c>
-      <c r="C50" s="295"/>
-      <c r="D50" s="295"/>
+      <c r="C50" s="274"/>
+      <c r="D50" s="274"/>
       <c r="E50" s="206"/>
       <c r="F50" s="28"/>
       <c r="J50" s="202"/>
@@ -3349,10 +3353,10 @@
       <c r="J51" s="202"/>
     </row>
     <row r="52" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="268"/>
-      <c r="B52" s="269"/>
-      <c r="C52" s="270"/>
-      <c r="D52" s="271"/>
+      <c r="A52" s="267"/>
+      <c r="B52" s="268"/>
+      <c r="C52" s="269"/>
+      <c r="D52" s="338"/>
       <c r="E52" s="206"/>
       <c r="F52" s="28"/>
       <c r="J52" s="202"/>
@@ -3385,8 +3389,8 @@
       <c r="A56" s="18"/>
       <c r="B56" s="122"/>
       <c r="C56" s="37"/>
-      <c r="D56" s="272"/>
-      <c r="E56" s="272"/>
+      <c r="D56" s="270"/>
+      <c r="E56" s="270"/>
       <c r="F56" s="214"/>
     </row>
     <row r="57" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -3401,19 +3405,6 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="B46:D46"/>
-    <mergeCell ref="B50:D50"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="A42:B42"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="A45:D45"/>
-    <mergeCell ref="A25:C25"/>
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="A38:C38"/>
-    <mergeCell ref="A44:C44"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="D7:F7"/>
@@ -3430,6 +3421,19 @@
     <mergeCell ref="A16:C16"/>
     <mergeCell ref="A33:C33"/>
     <mergeCell ref="A21:C21"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="B50:D50"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="A45:D45"/>
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="A44:C44"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.25" header="0.3" footer="0.3"/>
   <pageSetup scale="69" fitToHeight="0" orientation="portrait" r:id="rId1"/>
@@ -3455,14 +3459,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="23.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="309" t="s">
+      <c r="A1" s="307" t="s">
         <v>288</v>
       </c>
-      <c r="B1" s="309"/>
-      <c r="C1" s="309"/>
-      <c r="D1" s="309"/>
-      <c r="E1" s="309"/>
-      <c r="F1" s="309"/>
+      <c r="B1" s="307"/>
+      <c r="C1" s="307"/>
+      <c r="D1" s="307"/>
+      <c r="E1" s="307"/>
+      <c r="F1" s="307"/>
     </row>
     <row r="2" spans="1:9" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="128"/>
@@ -3867,12 +3871,12 @@
       <c r="P25" s="18"/>
     </row>
     <row r="26" spans="1:16" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="310"/>
-      <c r="B26" s="310"/>
-      <c r="C26" s="310"/>
-      <c r="D26" s="310"/>
-      <c r="E26" s="310"/>
-      <c r="F26" s="310"/>
+      <c r="A26" s="308"/>
+      <c r="B26" s="308"/>
+      <c r="C26" s="308"/>
+      <c r="D26" s="308"/>
+      <c r="E26" s="308"/>
+      <c r="F26" s="308"/>
     </row>
     <row r="27" spans="1:16" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="135" t="s">
@@ -3966,11 +3970,11 @@
       <c r="A34" s="157" t="s">
         <v>238</v>
       </c>
-      <c r="B34" s="310"/>
-      <c r="C34" s="310"/>
-      <c r="D34" s="310"/>
-      <c r="E34" s="310"/>
-      <c r="F34" s="310"/>
+      <c r="B34" s="308"/>
+      <c r="C34" s="308"/>
+      <c r="D34" s="308"/>
+      <c r="E34" s="308"/>
+      <c r="F34" s="308"/>
       <c r="K34" s="29"/>
       <c r="L34" s="18"/>
     </row>
@@ -4101,12 +4105,12 @@
       <c r="AU38" s="106"/>
     </row>
     <row r="39" spans="1:47" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="311"/>
-      <c r="B39" s="311"/>
-      <c r="C39" s="311"/>
-      <c r="D39" s="311"/>
-      <c r="E39" s="311"/>
-      <c r="F39" s="311"/>
+      <c r="A39" s="309"/>
+      <c r="B39" s="309"/>
+      <c r="C39" s="309"/>
+      <c r="D39" s="309"/>
+      <c r="E39" s="309"/>
+      <c r="F39" s="309"/>
     </row>
     <row r="40" spans="1:47" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="165" t="s">
@@ -4260,12 +4264,12 @@
       <c r="F50" s="139"/>
     </row>
     <row r="51" spans="1:6" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="311"/>
-      <c r="B51" s="311"/>
-      <c r="C51" s="311"/>
-      <c r="D51" s="311"/>
-      <c r="E51" s="311"/>
-      <c r="F51" s="311"/>
+      <c r="A51" s="309"/>
+      <c r="B51" s="309"/>
+      <c r="C51" s="309"/>
+      <c r="D51" s="309"/>
+      <c r="E51" s="309"/>
+      <c r="F51" s="309"/>
     </row>
     <row r="52" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="132" t="s">
@@ -4502,14 +4506,14 @@
       <c r="AU74" s="29"/>
     </row>
     <row r="75" spans="1:47" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A75" s="306" t="s">
+      <c r="A75" s="304" t="s">
         <v>75</v>
       </c>
-      <c r="B75" s="306"/>
-      <c r="C75" s="306"/>
-      <c r="D75" s="306"/>
-      <c r="E75" s="306"/>
-      <c r="F75" s="306"/>
+      <c r="B75" s="304"/>
+      <c r="C75" s="304"/>
+      <c r="D75" s="304"/>
+      <c r="E75" s="304"/>
+      <c r="F75" s="304"/>
     </row>
     <row r="76" spans="1:47" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76" s="143" t="s">
@@ -4566,20 +4570,20 @@
       <c r="F80" s="177"/>
     </row>
     <row r="81" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A81" s="306" t="s">
+      <c r="A81" s="304" t="s">
         <v>68</v>
       </c>
-      <c r="B81" s="307" t="s">
+      <c r="B81" s="305" t="s">
         <v>3</v>
       </c>
-      <c r="C81" s="307"/>
-      <c r="E81" s="308" t="s">
+      <c r="C81" s="305"/>
+      <c r="E81" s="306" t="s">
         <v>4</v>
       </c>
-      <c r="F81" s="308"/>
+      <c r="F81" s="306"/>
     </row>
     <row r="82" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A82" s="306"/>
+      <c r="A82" s="304"/>
       <c r="B82" s="149" t="s">
         <v>52</v>
       </c>
@@ -4895,14 +4899,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="23.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="309" t="s">
+      <c r="A1" s="307" t="s">
         <v>235</v>
       </c>
-      <c r="B1" s="309"/>
-      <c r="C1" s="309"/>
-      <c r="D1" s="309"/>
-      <c r="E1" s="309"/>
-      <c r="F1" s="309"/>
+      <c r="B1" s="307"/>
+      <c r="C1" s="307"/>
+      <c r="D1" s="307"/>
+      <c r="E1" s="307"/>
+      <c r="F1" s="307"/>
     </row>
     <row r="2" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="128"/>
@@ -5296,12 +5300,12 @@
       <c r="F25" s="156"/>
     </row>
     <row r="26" spans="1:16" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="310"/>
-      <c r="B26" s="310"/>
-      <c r="C26" s="310"/>
-      <c r="D26" s="310"/>
-      <c r="E26" s="310"/>
-      <c r="F26" s="310"/>
+      <c r="A26" s="308"/>
+      <c r="B26" s="308"/>
+      <c r="C26" s="308"/>
+      <c r="D26" s="308"/>
+      <c r="E26" s="308"/>
+      <c r="F26" s="308"/>
     </row>
     <row r="27" spans="1:16" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="135" t="s">
@@ -5402,11 +5406,11 @@
       <c r="A34" s="157" t="s">
         <v>238</v>
       </c>
-      <c r="B34" s="310"/>
-      <c r="C34" s="310"/>
-      <c r="D34" s="310"/>
-      <c r="E34" s="310"/>
-      <c r="F34" s="310"/>
+      <c r="B34" s="308"/>
+      <c r="C34" s="308"/>
+      <c r="D34" s="308"/>
+      <c r="E34" s="308"/>
+      <c r="F34" s="308"/>
     </row>
     <row r="35" spans="1:47" ht="0.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="157"/>
@@ -5531,12 +5535,12 @@
       <c r="F38" s="164"/>
     </row>
     <row r="39" spans="1:47" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="311"/>
-      <c r="B39" s="311"/>
-      <c r="C39" s="311"/>
-      <c r="D39" s="311"/>
-      <c r="E39" s="311"/>
-      <c r="F39" s="311"/>
+      <c r="A39" s="309"/>
+      <c r="B39" s="309"/>
+      <c r="C39" s="309"/>
+      <c r="D39" s="309"/>
+      <c r="E39" s="309"/>
+      <c r="F39" s="309"/>
     </row>
     <row r="40" spans="1:47" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="165" t="s">
@@ -5689,12 +5693,12 @@
       <c r="F50" s="139"/>
     </row>
     <row r="51" spans="1:6" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="311"/>
-      <c r="B51" s="311"/>
-      <c r="C51" s="311"/>
-      <c r="D51" s="311"/>
-      <c r="E51" s="311"/>
-      <c r="F51" s="311"/>
+      <c r="A51" s="309"/>
+      <c r="B51" s="309"/>
+      <c r="C51" s="309"/>
+      <c r="D51" s="309"/>
+      <c r="E51" s="309"/>
+      <c r="F51" s="309"/>
     </row>
     <row r="52" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="132" t="s">
@@ -5984,14 +5988,14 @@
       <c r="F74" s="140"/>
     </row>
     <row r="75" spans="1:47" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A75" s="306" t="s">
+      <c r="A75" s="304" t="s">
         <v>75</v>
       </c>
-      <c r="B75" s="306"/>
-      <c r="C75" s="306"/>
-      <c r="D75" s="306"/>
-      <c r="E75" s="306"/>
-      <c r="F75" s="306"/>
+      <c r="B75" s="304"/>
+      <c r="C75" s="304"/>
+      <c r="D75" s="304"/>
+      <c r="E75" s="304"/>
+      <c r="F75" s="304"/>
     </row>
     <row r="76" spans="1:47" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76" s="176">
@@ -6048,20 +6052,20 @@
       <c r="F80" s="177"/>
     </row>
     <row r="81" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A81" s="306" t="s">
+      <c r="A81" s="304" t="s">
         <v>68</v>
       </c>
-      <c r="B81" s="307" t="s">
+      <c r="B81" s="305" t="s">
         <v>3</v>
       </c>
-      <c r="C81" s="307"/>
-      <c r="E81" s="308" t="s">
+      <c r="C81" s="305"/>
+      <c r="E81" s="306" t="s">
         <v>4</v>
       </c>
-      <c r="F81" s="308"/>
+      <c r="F81" s="306"/>
     </row>
     <row r="82" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A82" s="306"/>
+      <c r="A82" s="304"/>
       <c r="B82" s="149" t="s">
         <v>52</v>
       </c>
@@ -6323,14 +6327,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="23.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="314" t="s">
+      <c r="A1" s="323" t="s">
         <v>207</v>
       </c>
-      <c r="B1" s="314"/>
-      <c r="C1" s="314"/>
-      <c r="D1" s="314"/>
-      <c r="E1" s="314"/>
-      <c r="F1" s="314"/>
+      <c r="B1" s="323"/>
+      <c r="C1" s="323"/>
+      <c r="D1" s="323"/>
+      <c r="E1" s="323"/>
+      <c r="F1" s="323"/>
     </row>
     <row r="2" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2"/>
@@ -6746,12 +6750,12 @@
       <c r="G25" s="1"/>
     </row>
     <row r="26" spans="1:7" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="315"/>
-      <c r="B26" s="316"/>
-      <c r="C26" s="316"/>
-      <c r="D26" s="316"/>
-      <c r="E26" s="316"/>
-      <c r="F26" s="316"/>
+      <c r="A26" s="324"/>
+      <c r="B26" s="325"/>
+      <c r="C26" s="325"/>
+      <c r="D26" s="325"/>
+      <c r="E26" s="325"/>
+      <c r="F26" s="325"/>
       <c r="G26" s="1"/>
     </row>
     <row r="27" spans="1:7" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -6834,23 +6838,23 @@
       <c r="G32" s="1"/>
     </row>
     <row r="33" spans="1:7" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="317"/>
-      <c r="B33" s="312"/>
-      <c r="C33" s="312"/>
-      <c r="D33" s="312"/>
-      <c r="E33" s="312"/>
-      <c r="F33" s="313"/>
+      <c r="A33" s="326"/>
+      <c r="B33" s="321"/>
+      <c r="C33" s="321"/>
+      <c r="D33" s="321"/>
+      <c r="E33" s="321"/>
+      <c r="F33" s="322"/>
       <c r="G33" s="1"/>
     </row>
     <row r="34" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="109" t="s">
         <v>36</v>
       </c>
-      <c r="B34" s="312"/>
-      <c r="C34" s="312"/>
-      <c r="D34" s="312"/>
-      <c r="E34" s="312"/>
-      <c r="F34" s="313"/>
+      <c r="B34" s="321"/>
+      <c r="C34" s="321"/>
+      <c r="D34" s="321"/>
+      <c r="E34" s="321"/>
+      <c r="F34" s="322"/>
       <c r="G34" s="1"/>
     </row>
     <row r="35" spans="1:7" s="106" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.35">
@@ -6889,12 +6893,12 @@
       <c r="G37" s="1"/>
     </row>
     <row r="38" spans="1:7" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="318"/>
-      <c r="B38" s="319"/>
-      <c r="C38" s="319"/>
-      <c r="D38" s="319"/>
-      <c r="E38" s="319"/>
-      <c r="F38" s="320"/>
+      <c r="A38" s="310"/>
+      <c r="B38" s="311"/>
+      <c r="C38" s="311"/>
+      <c r="D38" s="311"/>
+      <c r="E38" s="311"/>
+      <c r="F38" s="312"/>
       <c r="G38" s="1"/>
     </row>
     <row r="39" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
@@ -7059,12 +7063,12 @@
       <c r="G49" s="1"/>
     </row>
     <row r="50" spans="1:7" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="318"/>
-      <c r="B50" s="319"/>
-      <c r="C50" s="319"/>
-      <c r="D50" s="319"/>
-      <c r="E50" s="319"/>
-      <c r="F50" s="320"/>
+      <c r="A50" s="310"/>
+      <c r="B50" s="311"/>
+      <c r="C50" s="311"/>
+      <c r="D50" s="311"/>
+      <c r="E50" s="311"/>
+      <c r="F50" s="312"/>
       <c r="G50" s="1"/>
     </row>
     <row r="51" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
@@ -7255,14 +7259,14 @@
       <c r="G71" s="1"/>
     </row>
     <row r="72" spans="1:15" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A72" s="321" t="s">
+      <c r="A72" s="313" t="s">
         <v>75</v>
       </c>
-      <c r="B72" s="322"/>
-      <c r="C72" s="322"/>
-      <c r="D72" s="322"/>
-      <c r="E72" s="322"/>
-      <c r="F72" s="323"/>
+      <c r="B72" s="314"/>
+      <c r="C72" s="314"/>
+      <c r="D72" s="314"/>
+      <c r="E72" s="314"/>
+      <c r="F72" s="315"/>
       <c r="G72" s="1"/>
     </row>
     <row r="73" spans="1:15" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -7332,21 +7336,21 @@
       <c r="G77" s="1"/>
     </row>
     <row r="78" spans="1:15" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A78" s="324" t="s">
+      <c r="A78" s="316" t="s">
         <v>68</v>
       </c>
-      <c r="B78" s="326" t="s">
+      <c r="B78" s="318" t="s">
         <v>3</v>
       </c>
-      <c r="C78" s="326"/>
-      <c r="E78" s="327" t="s">
+      <c r="C78" s="318"/>
+      <c r="E78" s="319" t="s">
         <v>4</v>
       </c>
-      <c r="F78" s="328"/>
+      <c r="F78" s="320"/>
       <c r="G78" s="1"/>
     </row>
     <row r="79" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A79" s="325"/>
+      <c r="A79" s="317"/>
       <c r="B79" s="52" t="s">
         <v>52</v>
       </c>
@@ -7578,16 +7582,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B34:F34"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A38:F38"/>
     <mergeCell ref="A50:F50"/>
     <mergeCell ref="A72:F72"/>
     <mergeCell ref="A78:A79"/>
     <mergeCell ref="B78:C78"/>
     <mergeCell ref="E78:F78"/>
-    <mergeCell ref="B34:F34"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A26:F26"/>
-    <mergeCell ref="A33:F33"/>
-    <mergeCell ref="A38:F38"/>
   </mergeCells>
   <printOptions horizontalCentered="1" gridLines="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7618,14 +7622,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="23.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="314" t="s">
+      <c r="A1" s="323" t="s">
         <v>185</v>
       </c>
-      <c r="B1" s="314"/>
-      <c r="C1" s="314"/>
-      <c r="D1" s="314"/>
-      <c r="E1" s="314"/>
-      <c r="F1" s="314"/>
+      <c r="B1" s="323"/>
+      <c r="C1" s="323"/>
+      <c r="D1" s="323"/>
+      <c r="E1" s="323"/>
+      <c r="F1" s="323"/>
     </row>
     <row r="2" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2"/>
@@ -7895,11 +7899,11 @@
       <c r="A18" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="B18" s="329"/>
-      <c r="C18" s="327"/>
-      <c r="D18" s="327"/>
-      <c r="E18" s="327"/>
-      <c r="F18" s="328"/>
+      <c r="B18" s="327"/>
+      <c r="C18" s="319"/>
+      <c r="D18" s="319"/>
+      <c r="E18" s="319"/>
+      <c r="F18" s="320"/>
       <c r="G18" s="1"/>
     </row>
     <row r="19" spans="1:7" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -7986,12 +7990,12 @@
       <c r="G22" s="1"/>
     </row>
     <row r="23" spans="1:7" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="315"/>
-      <c r="B23" s="316"/>
-      <c r="C23" s="316"/>
-      <c r="D23" s="316"/>
-      <c r="E23" s="316"/>
-      <c r="F23" s="316"/>
+      <c r="A23" s="324"/>
+      <c r="B23" s="325"/>
+      <c r="C23" s="325"/>
+      <c r="D23" s="325"/>
+      <c r="E23" s="325"/>
+      <c r="F23" s="325"/>
       <c r="G23" s="1"/>
     </row>
     <row r="24" spans="1:7" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -8018,11 +8022,11 @@
       <c r="A25" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="B25" s="329"/>
-      <c r="C25" s="327"/>
-      <c r="D25" s="327"/>
-      <c r="E25" s="327"/>
-      <c r="F25" s="328"/>
+      <c r="B25" s="327"/>
+      <c r="C25" s="319"/>
+      <c r="D25" s="319"/>
+      <c r="E25" s="319"/>
+      <c r="F25" s="320"/>
       <c r="G25" s="1"/>
     </row>
     <row r="26" spans="1:7" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -8126,23 +8130,23 @@
       <c r="G30" s="1"/>
     </row>
     <row r="31" spans="1:7" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="317"/>
-      <c r="B31" s="312"/>
-      <c r="C31" s="312"/>
-      <c r="D31" s="312"/>
-      <c r="E31" s="312"/>
-      <c r="F31" s="313"/>
+      <c r="A31" s="326"/>
+      <c r="B31" s="321"/>
+      <c r="C31" s="321"/>
+      <c r="D31" s="321"/>
+      <c r="E31" s="321"/>
+      <c r="F31" s="322"/>
       <c r="G31" s="1"/>
     </row>
     <row r="32" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="B32" s="312"/>
-      <c r="C32" s="312"/>
-      <c r="D32" s="312"/>
-      <c r="E32" s="312"/>
-      <c r="F32" s="313"/>
+      <c r="B32" s="321"/>
+      <c r="C32" s="321"/>
+      <c r="D32" s="321"/>
+      <c r="E32" s="321"/>
+      <c r="F32" s="322"/>
       <c r="G32" s="1"/>
     </row>
     <row r="33" spans="1:7" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -8191,12 +8195,12 @@
       <c r="G35" s="1"/>
     </row>
     <row r="36" spans="1:7" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="318"/>
-      <c r="B36" s="319"/>
-      <c r="C36" s="319"/>
-      <c r="D36" s="319"/>
-      <c r="E36" s="319"/>
-      <c r="F36" s="320"/>
+      <c r="A36" s="310"/>
+      <c r="B36" s="311"/>
+      <c r="C36" s="311"/>
+      <c r="D36" s="311"/>
+      <c r="E36" s="311"/>
+      <c r="F36" s="312"/>
       <c r="G36" s="1"/>
     </row>
     <row r="37" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
@@ -8361,12 +8365,12 @@
       <c r="G47" s="1"/>
     </row>
     <row r="48" spans="1:7" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="318"/>
-      <c r="B48" s="319"/>
-      <c r="C48" s="319"/>
-      <c r="D48" s="319"/>
-      <c r="E48" s="319"/>
-      <c r="F48" s="320"/>
+      <c r="A48" s="310"/>
+      <c r="B48" s="311"/>
+      <c r="C48" s="311"/>
+      <c r="D48" s="311"/>
+      <c r="E48" s="311"/>
+      <c r="F48" s="312"/>
       <c r="G48" s="1"/>
     </row>
     <row r="49" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.35">
@@ -8572,14 +8576,14 @@
       <c r="G69" s="1"/>
     </row>
     <row r="70" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A70" s="321" t="s">
+      <c r="A70" s="313" t="s">
         <v>75</v>
       </c>
-      <c r="B70" s="322"/>
-      <c r="C70" s="322"/>
-      <c r="D70" s="322"/>
-      <c r="E70" s="322"/>
-      <c r="F70" s="323"/>
+      <c r="B70" s="314"/>
+      <c r="C70" s="314"/>
+      <c r="D70" s="314"/>
+      <c r="E70" s="314"/>
+      <c r="F70" s="315"/>
       <c r="G70" s="1"/>
     </row>
     <row r="71" spans="1:7" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -8655,21 +8659,21 @@
       <c r="G76" s="1"/>
     </row>
     <row r="77" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A77" s="324" t="s">
+      <c r="A77" s="316" t="s">
         <v>68</v>
       </c>
-      <c r="B77" s="326" t="s">
+      <c r="B77" s="318" t="s">
         <v>3</v>
       </c>
-      <c r="C77" s="326"/>
-      <c r="E77" s="327" t="s">
+      <c r="C77" s="318"/>
+      <c r="E77" s="319" t="s">
         <v>4</v>
       </c>
-      <c r="F77" s="328"/>
+      <c r="F77" s="320"/>
       <c r="G77" s="1"/>
     </row>
     <row r="78" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A78" s="325"/>
+      <c r="A78" s="317"/>
       <c r="B78" s="52" t="s">
         <v>52</v>
       </c>
@@ -8978,18 +8982,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A36:F36"/>
+    <mergeCell ref="A48:F48"/>
+    <mergeCell ref="A70:F70"/>
+    <mergeCell ref="A77:A78"/>
+    <mergeCell ref="B77:C77"/>
+    <mergeCell ref="E77:F77"/>
     <mergeCell ref="B32:F32"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B18:F18"/>
     <mergeCell ref="A23:F23"/>
     <mergeCell ref="B25:F25"/>
     <mergeCell ref="A31:F31"/>
-    <mergeCell ref="A36:F36"/>
-    <mergeCell ref="A48:F48"/>
-    <mergeCell ref="A70:F70"/>
-    <mergeCell ref="A77:A78"/>
-    <mergeCell ref="B77:C77"/>
-    <mergeCell ref="E77:F77"/>
   </mergeCells>
   <printOptions horizontalCentered="1" gridLines="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9017,14 +9021,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="23.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="314" t="s">
+      <c r="A1" s="323" t="s">
         <v>79</v>
       </c>
-      <c r="B1" s="314"/>
-      <c r="C1" s="314"/>
-      <c r="D1" s="314"/>
-      <c r="E1" s="314"/>
-      <c r="F1" s="314"/>
+      <c r="B1" s="323"/>
+      <c r="C1" s="323"/>
+      <c r="D1" s="323"/>
+      <c r="E1" s="323"/>
+      <c r="F1" s="323"/>
     </row>
     <row r="2" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2"/>
@@ -9271,11 +9275,11 @@
       <c r="A16" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="B16" s="329"/>
-      <c r="C16" s="327"/>
-      <c r="D16" s="327"/>
-      <c r="E16" s="327"/>
-      <c r="F16" s="328"/>
+      <c r="B16" s="327"/>
+      <c r="C16" s="319"/>
+      <c r="D16" s="319"/>
+      <c r="E16" s="319"/>
+      <c r="F16" s="320"/>
       <c r="G16" s="1"/>
     </row>
     <row r="17" spans="1:7" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -9319,12 +9323,12 @@
       <c r="G20" s="1"/>
     </row>
     <row r="21" spans="1:7" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="315"/>
-      <c r="B21" s="316"/>
-      <c r="C21" s="316"/>
-      <c r="D21" s="316"/>
-      <c r="E21" s="316"/>
-      <c r="F21" s="316"/>
+      <c r="A21" s="324"/>
+      <c r="B21" s="325"/>
+      <c r="C21" s="325"/>
+      <c r="D21" s="325"/>
+      <c r="E21" s="325"/>
+      <c r="F21" s="325"/>
       <c r="G21" s="1"/>
     </row>
     <row r="22" spans="1:7" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -9354,11 +9358,11 @@
       <c r="A23" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="B23" s="329"/>
-      <c r="C23" s="327"/>
-      <c r="D23" s="327"/>
-      <c r="E23" s="327"/>
-      <c r="F23" s="328"/>
+      <c r="B23" s="327"/>
+      <c r="C23" s="319"/>
+      <c r="D23" s="319"/>
+      <c r="E23" s="319"/>
+      <c r="F23" s="320"/>
       <c r="G23" s="1"/>
     </row>
     <row r="24" spans="1:7" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -9445,23 +9449,23 @@
       <c r="G28" s="1"/>
     </row>
     <row r="29" spans="1:7" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="317"/>
-      <c r="B29" s="312"/>
-      <c r="C29" s="312"/>
-      <c r="D29" s="312"/>
-      <c r="E29" s="312"/>
-      <c r="F29" s="313"/>
+      <c r="A29" s="326"/>
+      <c r="B29" s="321"/>
+      <c r="C29" s="321"/>
+      <c r="D29" s="321"/>
+      <c r="E29" s="321"/>
+      <c r="F29" s="322"/>
       <c r="G29" s="1"/>
     </row>
     <row r="30" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="B30" s="312"/>
-      <c r="C30" s="312"/>
-      <c r="D30" s="312"/>
-      <c r="E30" s="312"/>
-      <c r="F30" s="313"/>
+      <c r="B30" s="321"/>
+      <c r="C30" s="321"/>
+      <c r="D30" s="321"/>
+      <c r="E30" s="321"/>
+      <c r="F30" s="322"/>
       <c r="G30" s="1"/>
     </row>
     <row r="31" spans="1:7" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -9498,12 +9502,12 @@
       <c r="G33" s="1"/>
     </row>
     <row r="34" spans="1:7" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="318"/>
-      <c r="B34" s="319"/>
-      <c r="C34" s="319"/>
-      <c r="D34" s="319"/>
-      <c r="E34" s="319"/>
-      <c r="F34" s="320"/>
+      <c r="A34" s="310"/>
+      <c r="B34" s="311"/>
+      <c r="C34" s="311"/>
+      <c r="D34" s="311"/>
+      <c r="E34" s="311"/>
+      <c r="F34" s="312"/>
       <c r="G34" s="1"/>
     </row>
     <row r="35" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
@@ -9608,12 +9612,12 @@
       <c r="G41" s="1"/>
     </row>
     <row r="42" spans="1:7" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="318"/>
-      <c r="B42" s="319"/>
-      <c r="C42" s="319"/>
-      <c r="D42" s="319"/>
-      <c r="E42" s="319"/>
-      <c r="F42" s="320"/>
+      <c r="A42" s="310"/>
+      <c r="B42" s="311"/>
+      <c r="C42" s="311"/>
+      <c r="D42" s="311"/>
+      <c r="E42" s="311"/>
+      <c r="F42" s="312"/>
       <c r="G42" s="1"/>
     </row>
     <row r="43" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
@@ -9814,14 +9818,14 @@
       <c r="G63" s="1"/>
     </row>
     <row r="64" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A64" s="321" t="s">
+      <c r="A64" s="313" t="s">
         <v>75</v>
       </c>
-      <c r="B64" s="322"/>
-      <c r="C64" s="322"/>
-      <c r="D64" s="322"/>
-      <c r="E64" s="322"/>
-      <c r="F64" s="323"/>
+      <c r="B64" s="314"/>
+      <c r="C64" s="314"/>
+      <c r="D64" s="314"/>
+      <c r="E64" s="314"/>
+      <c r="F64" s="315"/>
       <c r="G64" s="1"/>
     </row>
     <row r="65" spans="1:7" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -9897,21 +9901,21 @@
       <c r="G70" s="1"/>
     </row>
     <row r="71" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A71" s="324" t="s">
+      <c r="A71" s="316" t="s">
         <v>68</v>
       </c>
-      <c r="B71" s="326" t="s">
+      <c r="B71" s="318" t="s">
         <v>3</v>
       </c>
-      <c r="C71" s="326"/>
-      <c r="E71" s="327" t="s">
+      <c r="C71" s="318"/>
+      <c r="E71" s="319" t="s">
         <v>4</v>
       </c>
-      <c r="F71" s="328"/>
+      <c r="F71" s="320"/>
       <c r="G71" s="1"/>
     </row>
     <row r="72" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A72" s="325"/>
+      <c r="A72" s="317"/>
       <c r="B72" s="52" t="s">
         <v>52</v>
       </c>
@@ -10229,13 +10233,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="330" t="s">
+      <c r="A1" s="328" t="s">
         <v>99</v>
       </c>
-      <c r="B1" s="330"/>
-      <c r="C1" s="330"/>
-      <c r="D1" s="330"/>
-      <c r="E1" s="330"/>
+      <c r="B1" s="328"/>
+      <c r="C1" s="328"/>
+      <c r="D1" s="328"/>
+      <c r="E1" s="328"/>
     </row>
     <row r="2" spans="1:6" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2"/>
@@ -10443,13 +10447,13 @@
       <c r="F14" s="1"/>
     </row>
     <row r="15" spans="1:6" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="331" t="s">
+      <c r="A15" s="329" t="s">
         <v>33</v>
       </c>
-      <c r="B15" s="331"/>
-      <c r="C15" s="331"/>
-      <c r="D15" s="331"/>
-      <c r="E15" s="331"/>
+      <c r="B15" s="329"/>
+      <c r="C15" s="329"/>
+      <c r="D15" s="329"/>
+      <c r="E15" s="329"/>
       <c r="F15" s="1"/>
     </row>
     <row r="16" spans="1:6" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -10530,13 +10534,13 @@
       <c r="F19" s="1"/>
     </row>
     <row r="20" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="331" t="s">
+      <c r="A20" s="329" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="331"/>
-      <c r="C20" s="331"/>
-      <c r="D20" s="331"/>
-      <c r="E20" s="331"/>
+      <c r="B20" s="329"/>
+      <c r="C20" s="329"/>
+      <c r="D20" s="329"/>
+      <c r="E20" s="329"/>
       <c r="F20" s="1"/>
     </row>
     <row r="21" spans="1:6" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -10688,11 +10692,11 @@
       <c r="F30" s="1"/>
     </row>
     <row r="31" spans="1:6" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="318"/>
-      <c r="B31" s="319"/>
-      <c r="C31" s="319"/>
-      <c r="D31" s="319"/>
-      <c r="E31" s="320"/>
+      <c r="A31" s="310"/>
+      <c r="B31" s="311"/>
+      <c r="C31" s="311"/>
+      <c r="D31" s="311"/>
+      <c r="E31" s="312"/>
       <c r="F31" s="1"/>
     </row>
     <row r="32" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.35">
@@ -10786,11 +10790,11 @@
       <c r="F38" s="1"/>
     </row>
     <row r="39" spans="1:6" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="318"/>
-      <c r="B39" s="319"/>
-      <c r="C39" s="319"/>
-      <c r="D39" s="319"/>
-      <c r="E39" s="320"/>
+      <c r="A39" s="310"/>
+      <c r="B39" s="311"/>
+      <c r="C39" s="311"/>
+      <c r="D39" s="311"/>
+      <c r="E39" s="312"/>
       <c r="F39" s="1"/>
     </row>
     <row r="40" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.35">
@@ -10996,13 +11000,13 @@
       <c r="F61" s="1"/>
     </row>
     <row r="62" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A62" s="321" t="s">
+      <c r="A62" s="313" t="s">
         <v>124</v>
       </c>
-      <c r="B62" s="322"/>
-      <c r="C62" s="322"/>
-      <c r="D62" s="322"/>
-      <c r="E62" s="323"/>
+      <c r="B62" s="314"/>
+      <c r="C62" s="314"/>
+      <c r="D62" s="314"/>
+      <c r="E62" s="315"/>
       <c r="F62" s="1"/>
     </row>
     <row r="63" spans="1:6" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -11080,13 +11084,13 @@
       <c r="F68" s="1"/>
     </row>
     <row r="69" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A69" s="324" t="s">
+      <c r="A69" s="316" t="s">
         <v>126</v>
       </c>
-      <c r="B69" s="326" t="s">
+      <c r="B69" s="318" t="s">
         <v>3</v>
       </c>
-      <c r="C69" s="326"/>
+      <c r="C69" s="318"/>
       <c r="D69" s="33" t="s">
         <v>4</v>
       </c>
@@ -11094,7 +11098,7 @@
       <c r="F69" s="1"/>
     </row>
     <row r="70" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A70" s="325"/>
+      <c r="A70" s="317"/>
       <c r="B70" s="52" t="s">
         <v>52</v>
       </c>
@@ -11371,34 +11375,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="27" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="333">
+      <c r="A1" s="332">
         <v>2017</v>
       </c>
-      <c r="B1" s="334"/>
-      <c r="C1" s="334"/>
-      <c r="D1" s="334"/>
-      <c r="E1" s="334"/>
-      <c r="F1" s="334"/>
-      <c r="G1" s="334"/>
-      <c r="H1" s="334"/>
-      <c r="I1" s="334"/>
-      <c r="J1" s="334"/>
-      <c r="K1" s="335"/>
+      <c r="B1" s="333"/>
+      <c r="C1" s="333"/>
+      <c r="D1" s="333"/>
+      <c r="E1" s="333"/>
+      <c r="F1" s="333"/>
+      <c r="G1" s="333"/>
+      <c r="H1" s="333"/>
+      <c r="I1" s="333"/>
+      <c r="J1" s="333"/>
+      <c r="K1" s="334"/>
     </row>
     <row r="2" spans="1:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="336" t="s">
+      <c r="A2" s="335" t="s">
         <v>133</v>
       </c>
-      <c r="B2" s="336"/>
-      <c r="C2" s="336"/>
-      <c r="D2" s="336"/>
-      <c r="E2" s="336"/>
-      <c r="F2" s="336"/>
-      <c r="G2" s="336"/>
-      <c r="H2" s="336"/>
-      <c r="I2" s="336"/>
-      <c r="J2" s="336"/>
-      <c r="K2" s="336"/>
+      <c r="B2" s="335"/>
+      <c r="C2" s="335"/>
+      <c r="D2" s="335"/>
+      <c r="E2" s="335"/>
+      <c r="F2" s="335"/>
+      <c r="G2" s="335"/>
+      <c r="H2" s="335"/>
+      <c r="I2" s="335"/>
+      <c r="J2" s="335"/>
+      <c r="K2" s="335"/>
       <c r="L2" s="66"/>
       <c r="M2" s="66"/>
       <c r="N2" s="66"/>
@@ -11422,10 +11426,10 @@
       <c r="E6" s="68">
         <v>0.13420000000000001</v>
       </c>
-      <c r="F6" s="337" t="s">
+      <c r="F6" s="336" t="s">
         <v>136</v>
       </c>
-      <c r="G6" s="337"/>
+      <c r="G6" s="336"/>
       <c r="L6" s="69"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
@@ -11438,10 +11442,10 @@
       <c r="E7" s="70">
         <v>0.37</v>
       </c>
-      <c r="F7" s="337" t="s">
+      <c r="F7" s="336" t="s">
         <v>138</v>
       </c>
-      <c r="G7" s="337"/>
+      <c r="G7" s="336"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="E8" s="70"/>
@@ -11652,10 +11656,10 @@
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A21" s="332" t="s">
+      <c r="A21" s="330" t="s">
         <v>159</v>
       </c>
-      <c r="B21" s="332"/>
+      <c r="B21" s="330"/>
       <c r="F21" s="29"/>
       <c r="K21" s="23"/>
     </row>
@@ -11808,10 +11812,10 @@
       <c r="P33" s="23"/>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A34" s="332" t="s">
+      <c r="A34" s="330" t="s">
         <v>169</v>
       </c>
-      <c r="B34" s="332"/>
+      <c r="B34" s="330"/>
       <c r="K34" s="79"/>
       <c r="P34" s="23"/>
     </row>
@@ -11860,12 +11864,12 @@
       <c r="G39" s="80"/>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A40" s="332" t="s">
+      <c r="A40" s="330" t="s">
         <v>174</v>
       </c>
-      <c r="B40" s="332"/>
-      <c r="C40" s="332"/>
-      <c r="D40" s="332"/>
+      <c r="B40" s="330"/>
+      <c r="C40" s="330"/>
+      <c r="D40" s="330"/>
       <c r="E40" s="28"/>
       <c r="G40" s="80"/>
       <c r="I40" s="80"/>
@@ -11888,10 +11892,10 @@
       <c r="K42" s="80"/>
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A43" s="332" t="s">
+      <c r="A43" s="330" t="s">
         <v>175</v>
       </c>
-      <c r="B43" s="332"/>
+      <c r="B43" s="330"/>
       <c r="C43" s="18">
         <v>39</v>
       </c>
@@ -11903,10 +11907,10 @@
       <c r="K43" s="80"/>
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A44" s="332" t="s">
+      <c r="A44" s="330" t="s">
         <v>177</v>
       </c>
-      <c r="B44" s="332"/>
+      <c r="B44" s="330"/>
       <c r="C44" s="18">
         <v>11</v>
       </c>
@@ -11918,10 +11922,10 @@
       <c r="K44" s="80"/>
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A45" s="332" t="s">
+      <c r="A45" s="330" t="s">
         <v>178</v>
       </c>
-      <c r="B45" s="332"/>
+      <c r="B45" s="330"/>
       <c r="C45" s="18">
         <v>16</v>
       </c>
@@ -11933,10 +11937,10 @@
       <c r="K45" s="80"/>
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A46" s="332" t="s">
+      <c r="A46" s="330" t="s">
         <v>179</v>
       </c>
-      <c r="B46" s="332"/>
+      <c r="B46" s="330"/>
       <c r="C46" s="18">
         <v>73</v>
       </c>
@@ -11948,10 +11952,10 @@
       <c r="K46" s="80"/>
     </row>
     <row r="47" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="332" t="s">
+      <c r="A47" s="330" t="s">
         <v>180</v>
       </c>
-      <c r="B47" s="332"/>
+      <c r="B47" s="330"/>
       <c r="C47" s="18">
         <v>71</v>
       </c>
@@ -11978,10 +11982,10 @@
       <c r="K49" s="80"/>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A50" s="332" t="s">
+      <c r="A50" s="330" t="s">
         <v>181</v>
       </c>
-      <c r="B50" s="332"/>
+      <c r="B50" s="330"/>
       <c r="C50" s="18">
         <v>17.399999999999999</v>
       </c>
@@ -12007,10 +12011,10 @@
       <c r="K52" s="80"/>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A53" s="338" t="s">
+      <c r="A53" s="331" t="s">
         <v>183</v>
       </c>
-      <c r="B53" s="338"/>
+      <c r="B53" s="331"/>
       <c r="C53" s="82">
         <v>16.73</v>
       </c>
@@ -12115,6 +12119,12 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="A21:B21"/>
     <mergeCell ref="A50:B50"/>
     <mergeCell ref="A53:B53"/>
     <mergeCell ref="A40:D40"/>
@@ -12123,12 +12133,6 @@
     <mergeCell ref="A45:B45"/>
     <mergeCell ref="A46:B46"/>
     <mergeCell ref="A47:B47"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="A21:B21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>